<commit_message>
Label the scenario workbook's Results sheet first
Results is the sheet the scenario workbook opens on. Row 1 now says it is an
illustrative scenario from stated assumptions, not a forecast or funding
conclusion, and that shares of trials are not probabilities; row 2 links to
About. The template is patched in place (rows shifted, frozen header moved)
and its manifest records the new row count and SHA-256.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/scenario_template.xlsx
+++ b/samples/scenario_template.xlsx
@@ -976,117 +976,53 @@
     <x:col min="11" max="11" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="40" customHeight="1">
-      <x:c r="A1" s="31" t="str">
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="56"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="55"/>
+    </x:row>
+    <x:row r="3" ht="40" customHeight="1">
+      <x:c r="A3" s="31" t="str">
         <x:v>Decision</x:v>
       </x:c>
-      <x:c r="B1" s="32" t="str">
+      <x:c r="B3" s="32" t="str">
         <x:v>Capex (USD, displayed in millions)</x:v>
       </x:c>
-      <x:c r="C1" s="32" t="str">
+      <x:c r="C3" s="32" t="str">
         <x:v>Dividends (USD, displayed in millions)</x:v>
       </x:c>
-      <x:c r="D1" s="32" t="str">
+      <x:c r="D3" s="32" t="str">
         <x:v>Revolver assumed usable</x:v>
       </x:c>
-      <x:c r="E1" s="32" t="str">
+      <x:c r="E3" s="32" t="str">
         <x:v>Mean ending cash (USD, displayed in millions)</x:v>
       </x:c>
-      <x:c r="F1" s="32" t="str">
+      <x:c r="F3" s="32" t="str">
         <x:v>Std dev (USD, displayed in millions)</x:v>
       </x:c>
-      <x:c r="G1" s="32" t="str">
+      <x:c r="G3" s="32" t="str">
         <x:v>10th percentile (USD, displayed in millions)</x:v>
       </x:c>
-      <x:c r="H1" s="32" t="str">
+      <x:c r="H3" s="32" t="str">
         <x:v>Median (USD, displayed in millions)</x:v>
       </x:c>
-      <x:c r="I1" s="32" t="str">
+      <x:c r="I3" s="32" t="str">
         <x:v>90th percentile (USD, displayed in millions)</x:v>
       </x:c>
-      <x:c r="J1" s="32" t="str">
+      <x:c r="J3" s="32" t="str">
         <x:v>Share of trials below zero</x:v>
       </x:c>
-      <x:c r="K1" s="33" t="str">
+      <x:c r="K3" s="33" t="str">
         <x:v>Average shortfall in trials below zero (USD, displayed in millions)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="32" customHeight="1">
-      <x:c r="A2" s="12" t="str">
-        <x:v>Capex at the TTM rate</x:v>
-      </x:c>
-      <x:c r="B2" s="13" t="n">
-        <x:v>75660000000</x:v>
-      </x:c>
-      <x:c r="C2" s="13" t="n">
-        <x:v>6260000000</x:v>
-      </x:c>
-      <x:c r="D2" s="14" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E2" s="13" t="n">
-        <x:v>-11232769857.50195</x:v>
-      </x:c>
-      <x:c r="F2" s="13" t="n">
-        <x:v>4172297711.8683176</x:v>
-      </x:c>
-      <x:c r="G2" s="13" t="n">
-        <x:v>-16628558782.73629</x:v>
-      </x:c>
-      <x:c r="H2" s="13" t="n">
-        <x:v>-11474076193.260605</x:v>
-      </x:c>
-      <x:c r="I2" s="13" t="n">
-        <x:v>-5579835245.119098</x:v>
-      </x:c>
-      <x:c r="J2" s="15" t="n">
-        <x:v>0.9948</x:v>
-      </x:c>
-      <x:c r="K2" s="16" t="n">
-        <x:v>11297149882.895933</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="40" customHeight="1">
-      <x:c r="A3" s="12" t="str">
-        <x:v>Capex at the TTM rate, revolver assumed usable</x:v>
-      </x:c>
-      <x:c r="B3" s="13" t="n">
-        <x:v>75660000000</x:v>
-      </x:c>
-      <x:c r="C3" s="13" t="n">
-        <x:v>6260000000</x:v>
-      </x:c>
-      <x:c r="D3" s="14" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="E3" s="13" t="n">
-        <x:v>-2401146269.8532047</x:v>
-      </x:c>
-      <x:c r="F3" s="13" t="n">
-        <x:v>2686931022.721906</x:v>
-      </x:c>
-      <x:c r="G3" s="13" t="n">
-        <x:v>-6628558782.73629</x:v>
-      </x:c>
-      <x:c r="H3" s="13" t="n">
-        <x:v>-1474076193.260604</x:v>
-      </x:c>
-      <x:c r="I3" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J3" s="15" t="n">
-        <x:v>0.6261</x:v>
-      </x:c>
-      <x:c r="K3" s="16" t="n">
-        <x:v>3844084197.182765</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="12" t="str">
-        <x:v>Capex at the fiscal 2026 level</x:v>
+        <x:v>Capex at the TTM rate</x:v>
       </x:c>
       <x:c r="B4" s="13" t="n">
-        <x:v>55663000000</x:v>
+        <x:v>75660000000</x:v>
       </x:c>
       <x:c r="C4" s="13" t="n">
         <x:v>6260000000</x:v>
@@ -1095,63 +1031,136 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E4" s="13" t="n">
-        <x:v>8764230142.49805</x:v>
+        <x:v>-11232769857.50195</x:v>
       </x:c>
       <x:c r="F4" s="13" t="n">
         <x:v>4172297711.8683176</x:v>
       </x:c>
       <x:c r="G4" s="13" t="n">
+        <x:v>-16628558782.73629</x:v>
+      </x:c>
+      <x:c r="H4" s="13" t="n">
+        <x:v>-11474076193.260605</x:v>
+      </x:c>
+      <x:c r="I4" s="13" t="n">
+        <x:v>-5579835245.119098</x:v>
+      </x:c>
+      <x:c r="J4" s="15" t="n">
+        <x:v>0.9948</x:v>
+      </x:c>
+      <x:c r="K4" s="16" t="n">
+        <x:v>11297149882.895933</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="40" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Capex at the TTM rate, revolver assumed usable</x:v>
+      </x:c>
+      <x:c r="B5" s="13" t="n">
+        <x:v>75660000000</x:v>
+      </x:c>
+      <x:c r="C5" s="13" t="n">
+        <x:v>6260000000</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E5" s="13" t="n">
+        <x:v>-2401146269.8532047</x:v>
+      </x:c>
+      <x:c r="F5" s="13" t="n">
+        <x:v>2686931022.721906</x:v>
+      </x:c>
+      <x:c r="G5" s="13" t="n">
+        <x:v>-6628558782.73629</x:v>
+      </x:c>
+      <x:c r="H5" s="13" t="n">
+        <x:v>-1474076193.260604</x:v>
+      </x:c>
+      <x:c r="I5" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J5" s="15" t="n">
+        <x:v>0.6261</x:v>
+      </x:c>
+      <x:c r="K5" s="16" t="n">
+        <x:v>3844084197.182765</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="32" customHeight="1">
+      <x:c r="A6" s="12" t="str">
+        <x:v>Capex at the fiscal 2026 level</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="n">
+        <x:v>55663000000</x:v>
+      </x:c>
+      <x:c r="C6" s="13" t="n">
+        <x:v>6260000000</x:v>
+      </x:c>
+      <x:c r="D6" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E6" s="13" t="n">
+        <x:v>8764230142.49805</x:v>
+      </x:c>
+      <x:c r="F6" s="13" t="n">
+        <x:v>4172297711.8683176</x:v>
+      </x:c>
+      <x:c r="G6" s="13" t="n">
         <x:v>3368441217.2637105</x:v>
       </x:c>
-      <x:c r="H4" s="13" t="n">
+      <x:c r="H6" s="13" t="n">
         <x:v>8522923806.739397</x:v>
       </x:c>
-      <x:c r="I4" s="13" t="n">
+      <x:c r="I6" s="13" t="n">
         <x:v>14417164754.880903</x:v>
       </x:c>
-      <x:c r="J4" s="15" t="n">
+      <x:c r="J6" s="15" t="n">
         <x:v>0.0023</x:v>
       </x:c>
-      <x:c r="K4" s="16" t="n">
+      <x:c r="K6" s="16" t="n">
         <x:v>300620628.9294267</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="40" customHeight="1">
-      <x:c r="A5" s="17" t="str">
+    <x:row r="7" ht="40" customHeight="1">
+      <x:c r="A7" s="17" t="str">
         <x:v>Capex at the fiscal 2026 level, revolver assumed usable</x:v>
       </x:c>
-      <x:c r="B5" s="18" t="n">
+      <x:c r="B7" s="18" t="n">
         <x:v>55663000000</x:v>
       </x:c>
-      <x:c r="C5" s="18" t="n">
+      <x:c r="C7" s="18" t="n">
         <x:v>6260000000</x:v>
       </x:c>
-      <x:c r="D5" s="19" t="str">
+      <x:c r="D7" s="19" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="E5" s="18" t="n">
+      <x:c r="E7" s="18" t="n">
         <x:v>8764921569.944588</x:v>
       </x:c>
-      <x:c r="F5" s="18" t="n">
+      <x:c r="F7" s="18" t="n">
         <x:v>4170807288.6858044</x:v>
       </x:c>
-      <x:c r="G5" s="18" t="n">
+      <x:c r="G7" s="18" t="n">
         <x:v>3368441217.2637105</x:v>
       </x:c>
-      <x:c r="H5" s="18" t="n">
+      <x:c r="H7" s="18" t="n">
         <x:v>8522923806.739397</x:v>
       </x:c>
-      <x:c r="I5" s="18" t="n">
+      <x:c r="I7" s="18" t="n">
         <x:v>14417164754.880903</x:v>
       </x:c>
-      <x:c r="J5" s="20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K5" s="21" t="n">
+      <x:c r="J7" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K7" s="21" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:hyperlinks>
+    <x:hyperlink ref="A2" location="'About'!A1" display="About"/>
+  </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>

</xml_diff>